<commit_message>
Mise à jour localisation Nodes
Corrections position des nodes:
- Entwaesserungstollen
- Quellteich
- Gischeren
Reste à faire: les arrivées d'eau dans le SonSto
</commit_message>
<xml_diff>
--- a/260508_Coord_nodes_SWMM.xlsx
+++ b/260508_Coord_nodes_SWMM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\ISSKA\Documents\GitHub\Twanntunnel_Hydraulic_SWMM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1491210-8CF9-47B7-90FF-30013887706B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4856495B-AE6B-413C-898E-CADCDE142681}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20385" windowHeight="11475" xr2:uid="{5560F17C-8740-4256-B354-A6A3ABF31B82}"/>
   </bookViews>
@@ -729,13 +729,13 @@
         <v>47</v>
       </c>
       <c r="B19">
-        <v>2578209</v>
+        <v>2578188</v>
       </c>
       <c r="C19">
-        <v>1215909</v>
+        <v>1215916</v>
       </c>
       <c r="D19" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -743,7 +743,7 @@
         <v>48</v>
       </c>
       <c r="B20">
-        <v>2578176</v>
+        <v>2578173</v>
       </c>
       <c r="C20">
         <v>1215879</v>
@@ -903,7 +903,7 @@
         <v>1215714</v>
       </c>
       <c r="D31" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -925,13 +925,13 @@
         <v>5</v>
       </c>
       <c r="B33">
-        <v>2578211</v>
+        <v>2578192</v>
       </c>
       <c r="C33">
-        <v>1215907</v>
+        <v>1215916</v>
       </c>
       <c r="D33" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -945,7 +945,7 @@
         <v>1215922</v>
       </c>
       <c r="D34" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -953,13 +953,13 @@
         <v>7</v>
       </c>
       <c r="B35">
-        <v>2578213</v>
+        <v>2578210</v>
       </c>
       <c r="C35">
-        <v>1215895</v>
+        <v>1215909</v>
       </c>
       <c r="D35" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Update SS3, SS4, SS5, SS6, etc.
Mise à jour des localisations, des géométries et des longueurs.
</commit_message>
<xml_diff>
--- a/260508_Coord_nodes_SWMM.xlsx
+++ b/260508_Coord_nodes_SWMM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\ISSKA\Documents\GitHub\Twanntunnel_Hydraulic_SWMM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4856495B-AE6B-413C-898E-CADCDE142681}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A585B224-074B-4281-A33D-F37B07E69FCB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20385" windowHeight="11475" xr2:uid="{5560F17C-8740-4256-B354-A6A3ABF31B82}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="50">
   <si>
     <t>Holiloch_sonde</t>
   </si>
@@ -112,6 +112,69 @@
   </si>
   <si>
     <t>SS1</t>
+  </si>
+  <si>
+    <t>TWT_Portail_Est</t>
+  </si>
+  <si>
+    <t>Chaussée</t>
+  </si>
+  <si>
+    <t>Radier</t>
+  </si>
+  <si>
+    <t>TWT_RebenWeg_61+575</t>
+  </si>
+  <si>
+    <t>TWT_Frauenchapf_61+380</t>
+  </si>
+  <si>
+    <t>TWT_Chrosweg_61+140</t>
+  </si>
+  <si>
+    <t>TWT_Hoole_61+020</t>
+  </si>
+  <si>
+    <t>TWT_Chrankwil_60+740</t>
+  </si>
+  <si>
+    <t>TWT_Branche_Est_Sonsto_60+540</t>
+  </si>
+  <si>
+    <t>TWT_Tschampet _60+650</t>
+  </si>
+  <si>
+    <t>TWT_Fensterstollen_60+375</t>
+  </si>
+  <si>
+    <t>TWT_Intersection_Sonsto_60+345</t>
+  </si>
+  <si>
+    <t>TWT_Acces_LT_60+110</t>
+  </si>
+  <si>
+    <t>TWT_Liaison_LT_59+738</t>
+  </si>
+  <si>
+    <t>SonSto_SS5</t>
+  </si>
+  <si>
+    <t>SonSto_SS3</t>
+  </si>
+  <si>
+    <t>Aval_Trappe</t>
+  </si>
+  <si>
+    <t>Amont_Trappe</t>
+  </si>
+  <si>
+    <t>SonSto_F</t>
+  </si>
+  <si>
+    <t>SonSto_SS6</t>
+  </si>
+  <si>
+    <t>SonSto_SS4</t>
   </si>
 </sst>
 </file>
@@ -466,7 +529,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{336D857F-22C8-4624-8585-90FCE8727574}">
-  <dimension ref="A1:D55"/>
+  <dimension ref="A1:F71"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="43.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -557,14 +620,14 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
-        <v>442</v>
+      <c r="A7" s="1" t="s">
+        <v>47</v>
       </c>
       <c r="B7">
-        <v>2578239</v>
+        <v>2578235</v>
       </c>
       <c r="C7">
-        <v>1215864</v>
+        <v>1215865</v>
       </c>
       <c r="D7" t="s">
         <v>26</v>
@@ -585,154 +648,151 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
-        <v>25</v>
+      <c r="A9" s="1" t="s">
+        <v>46</v>
       </c>
       <c r="B9">
-        <v>2578240</v>
+        <v>2578239</v>
       </c>
       <c r="C9">
-        <v>1215859</v>
-      </c>
-      <c r="D9" t="s">
-        <v>25</v>
+        <v>1215862</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="1">
+      <c r="A10" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B10">
+        <v>2578241</v>
+      </c>
+      <c r="C10">
+        <v>1215860</v>
+      </c>
+      <c r="D10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
         <v>30</v>
       </c>
-      <c r="B10">
+      <c r="B11">
         <v>2578252</v>
       </c>
-      <c r="C10">
+      <c r="C11">
         <v>1215847</v>
       </c>
-      <c r="D10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="D11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B11">
+      <c r="B12">
         <v>2578233</v>
       </c>
-      <c r="C11">
+      <c r="C12">
         <v>1215892</v>
       </c>
-      <c r="D11" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="1">
-        <v>34</v>
-      </c>
-      <c r="B12">
-        <v>2578051</v>
-      </c>
-      <c r="C12">
-        <v>1215607</v>
-      </c>
       <c r="D12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
+        <v>34</v>
+      </c>
+      <c r="B13">
+        <v>2578051</v>
+      </c>
+      <c r="C13">
+        <v>1215607</v>
+      </c>
+      <c r="D13" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
         <v>38</v>
       </c>
-      <c r="B13">
+      <c r="B14">
         <v>2578158</v>
       </c>
-      <c r="C13">
+      <c r="C14">
         <v>1215716</v>
       </c>
-      <c r="D13" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="D14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B14">
-        <v>2578248</v>
-      </c>
-      <c r="C14">
+      <c r="B15">
+        <v>2578247</v>
+      </c>
+      <c r="C15">
         <v>1215879</v>
       </c>
-      <c r="D14" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="1">
-        <v>40</v>
-      </c>
-      <c r="B15">
-        <v>2578259</v>
-      </c>
-      <c r="C15">
-        <v>1215858</v>
-      </c>
       <c r="D15" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
+        <v>40</v>
+      </c>
+      <c r="B16">
+        <v>2578259</v>
+      </c>
+      <c r="C16">
+        <v>1215858</v>
+      </c>
+      <c r="D16" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
         <v>41</v>
       </c>
-      <c r="B16">
+      <c r="B17">
         <v>2578210</v>
       </c>
-      <c r="C16">
+      <c r="C17">
         <v>1215870</v>
       </c>
-      <c r="D16" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+      <c r="D17" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B17">
+      <c r="B18">
         <v>2578171</v>
       </c>
-      <c r="C17">
+      <c r="C18">
         <v>1215878</v>
       </c>
-      <c r="D17" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="1">
-        <v>46</v>
-      </c>
-      <c r="B18">
+      <c r="D18" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19">
         <v>2578252</v>
       </c>
-      <c r="C18">
+      <c r="C19">
         <v>1215886</v>
-      </c>
-      <c r="D18" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="1">
-        <v>47</v>
-      </c>
-      <c r="B19">
-        <v>2578188</v>
-      </c>
-      <c r="C19">
-        <v>1215916</v>
       </c>
       <c r="D19" t="s">
         <v>26</v>
@@ -740,55 +800,55 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
+        <v>47</v>
+      </c>
+      <c r="B20">
+        <v>2578188</v>
+      </c>
+      <c r="C20">
+        <v>1215916</v>
+      </c>
+      <c r="D20" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
         <v>48</v>
       </c>
-      <c r="B20">
+      <c r="B21">
         <v>2578173</v>
       </c>
-      <c r="C20">
+      <c r="C21">
         <v>1215879</v>
       </c>
-      <c r="D20" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+      <c r="D21" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B21">
+      <c r="B22">
         <v>2578251</v>
       </c>
-      <c r="C21">
+      <c r="C22">
         <v>1215912</v>
       </c>
-      <c r="D21" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="1">
-        <v>49</v>
-      </c>
-      <c r="B22">
-        <v>2578248</v>
-      </c>
-      <c r="C22">
-        <v>1215880</v>
-      </c>
       <c r="D22" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B23">
-        <v>2578243</v>
+        <v>2578248</v>
       </c>
       <c r="C23">
-        <v>1215892</v>
+        <v>1215880</v>
       </c>
       <c r="D23" t="s">
         <v>25</v>
@@ -796,41 +856,41 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
+        <v>50</v>
+      </c>
+      <c r="B24">
+        <v>2578243</v>
+      </c>
+      <c r="C24">
+        <v>1215892</v>
+      </c>
+      <c r="D24" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
         <v>51</v>
       </c>
-      <c r="B24">
+      <c r="B25">
         <v>2578212</v>
       </c>
-      <c r="C24">
+      <c r="C25">
         <v>1215860</v>
       </c>
-      <c r="D24" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
+      <c r="D25" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B25">
+      <c r="B26">
         <v>2578165</v>
       </c>
-      <c r="C25">
+      <c r="C26">
         <v>1215931</v>
-      </c>
-      <c r="D25" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="1">
-        <v>52</v>
-      </c>
-      <c r="B26">
-        <v>2578146</v>
-      </c>
-      <c r="C26">
-        <v>1215780</v>
       </c>
       <c r="D26" t="s">
         <v>25</v>
@@ -838,13 +898,13 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B27">
-        <v>2578230</v>
+        <v>2578146</v>
       </c>
       <c r="C27">
-        <v>1215870</v>
+        <v>1215780</v>
       </c>
       <c r="D27" t="s">
         <v>25</v>
@@ -852,13 +912,13 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B28">
-        <v>2578250</v>
+        <v>2578230</v>
       </c>
       <c r="C28">
-        <v>1215883</v>
+        <v>1215870</v>
       </c>
       <c r="D28" t="s">
         <v>25</v>
@@ -866,13 +926,13 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B29">
-        <v>2578249</v>
+        <v>2578250</v>
       </c>
       <c r="C29">
-        <v>1215843</v>
+        <v>1215883</v>
       </c>
       <c r="D29" t="s">
         <v>25</v>
@@ -880,13 +940,13 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B30">
-        <v>2578156</v>
+        <v>2578249</v>
       </c>
       <c r="C30">
-        <v>1215910</v>
+        <v>1215843</v>
       </c>
       <c r="D30" t="s">
         <v>25</v>
@@ -894,55 +954,55 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
-        <v>2</v>
+        <v>57</v>
       </c>
       <c r="B31">
-        <v>2578030</v>
+        <v>2578156</v>
       </c>
       <c r="C31">
-        <v>1215714</v>
+        <v>1215910</v>
       </c>
       <c r="D31" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B32">
-        <v>2578040</v>
+        <v>2578030</v>
       </c>
       <c r="C32">
-        <v>1215610</v>
+        <v>1215714</v>
       </c>
       <c r="D32" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B33">
-        <v>2578192</v>
+        <v>2578040</v>
       </c>
       <c r="C33">
-        <v>1215916</v>
+        <v>1215610</v>
       </c>
       <c r="D33" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B34">
-        <v>2578186</v>
+        <v>2578192</v>
       </c>
       <c r="C34">
-        <v>1215922</v>
+        <v>1215916</v>
       </c>
       <c r="D34" t="s">
         <v>26</v>
@@ -950,27 +1010,27 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
+        <v>6</v>
+      </c>
+      <c r="B35">
+        <v>2578186</v>
+      </c>
+      <c r="C35">
+        <v>1215922</v>
+      </c>
+      <c r="D35" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
         <v>7</v>
       </c>
-      <c r="B35">
+      <c r="B36">
         <v>2578210</v>
       </c>
-      <c r="C35">
+      <c r="C36">
         <v>1215909</v>
-      </c>
-      <c r="D35" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B36">
-        <v>2578278</v>
-      </c>
-      <c r="C36">
-        <v>1215914</v>
       </c>
       <c r="D36" t="s">
         <v>26</v>
@@ -978,69 +1038,69 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B37">
+        <v>2578278</v>
+      </c>
+      <c r="C37">
+        <v>1215914</v>
+      </c>
+      <c r="D37" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B37">
+      <c r="B38">
         <v>2578261</v>
       </c>
-      <c r="C37">
+      <c r="C38">
         <v>1215889</v>
       </c>
-      <c r="D37" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="1">
-        <v>8</v>
-      </c>
-      <c r="B38">
-        <v>2578223</v>
-      </c>
-      <c r="C38">
-        <v>1215890</v>
-      </c>
       <c r="D38" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
+        <v>8</v>
+      </c>
+      <c r="B39">
+        <v>2578223</v>
+      </c>
+      <c r="C39">
+        <v>1215890</v>
+      </c>
+      <c r="D39" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="1">
         <v>10</v>
       </c>
-      <c r="B39">
+      <c r="B40">
         <v>2578244</v>
       </c>
-      <c r="C39">
+      <c r="C40">
         <v>1215877</v>
       </c>
-      <c r="D39" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B40">
-        <v>2578055</v>
-      </c>
-      <c r="C40">
-        <v>1215587</v>
-      </c>
       <c r="D40" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="B41">
-        <v>2578032</v>
+        <v>2578055</v>
       </c>
       <c r="C41">
-        <v>1215595</v>
+        <v>1215587</v>
       </c>
       <c r="D41" t="s">
         <v>26</v>
@@ -1048,13 +1108,13 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="B42">
-        <v>2578254</v>
+        <v>2578032</v>
       </c>
       <c r="C42">
-        <v>1215837</v>
+        <v>1215595</v>
       </c>
       <c r="D42" t="s">
         <v>26</v>
@@ -1062,13 +1122,13 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B43">
-        <v>2578235</v>
+        <v>2578254</v>
       </c>
       <c r="C43">
-        <v>1215889</v>
+        <v>1215837</v>
       </c>
       <c r="D43" t="s">
         <v>26</v>
@@ -1076,13 +1136,13 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B44">
-        <v>2578175</v>
+        <v>2578235</v>
       </c>
       <c r="C44">
-        <v>1215872</v>
+        <v>1215889</v>
       </c>
       <c r="D44" t="s">
         <v>26</v>
@@ -1090,13 +1150,13 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="B45">
-        <v>2578210</v>
+        <v>2578175</v>
       </c>
       <c r="C45">
-        <v>1215890</v>
+        <v>1215872</v>
       </c>
       <c r="D45" t="s">
         <v>26</v>
@@ -1104,13 +1164,13 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B46">
-        <v>2578244</v>
+        <v>2578210</v>
       </c>
       <c r="C46">
-        <v>1215830</v>
+        <v>1215890</v>
       </c>
       <c r="D46" t="s">
         <v>26</v>
@@ -1118,13 +1178,13 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B47">
-        <v>2578038</v>
+        <v>2578244</v>
       </c>
       <c r="C47">
-        <v>1215632</v>
+        <v>1215830</v>
       </c>
       <c r="D47" t="s">
         <v>26</v>
@@ -1132,77 +1192,343 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B48">
+        <v>2578038</v>
+      </c>
+      <c r="C48">
+        <v>1215632</v>
+      </c>
+      <c r="D48" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B48">
+      <c r="B49">
         <v>2578074</v>
       </c>
-      <c r="C48">
+      <c r="C49">
         <v>1215560</v>
       </c>
-      <c r="D48" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="1" t="s">
+      <c r="D49" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B49">
+      <c r="B50">
         <v>2578059</v>
       </c>
-      <c r="C49">
+      <c r="C50">
         <v>1215593</v>
       </c>
-      <c r="D49" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D50" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B51">
+        <v>2578260</v>
+      </c>
+      <c r="C51">
+        <v>1215893</v>
+      </c>
+      <c r="D51" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B52">
+        <v>2578277</v>
+      </c>
+      <c r="C52">
+        <v>1215915</v>
+      </c>
+      <c r="D52" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B53">
+        <v>2578254</v>
+      </c>
+      <c r="C53">
+        <v>1215885</v>
+      </c>
+      <c r="D53" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B54">
+        <v>2578249</v>
+      </c>
+      <c r="C54">
+        <v>1215879</v>
+      </c>
+      <c r="D54" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" s="1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="1" t="s">
+      <c r="E57" t="s">
+        <v>30</v>
+      </c>
+      <c r="F57" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B53">
+      <c r="B58">
         <v>2578983</v>
       </c>
-      <c r="C53">
+      <c r="C58">
         <v>1216295</v>
       </c>
-      <c r="D53">
+      <c r="D58">
         <v>436</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B54">
-        <v>2578265</v>
-      </c>
-      <c r="C54">
-        <v>1215898</v>
-      </c>
-      <c r="D54">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B59">
+        <v>2578361</v>
+      </c>
+      <c r="C59">
+        <v>1215967</v>
+      </c>
+      <c r="D59">
         <v>443</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B55">
-        <v>2578361</v>
-      </c>
-      <c r="C55">
-        <v>1215967</v>
-      </c>
-      <c r="D55">
-        <v>443</v>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B60">
+        <v>2579848</v>
+      </c>
+      <c r="C60">
+        <v>1216615</v>
+      </c>
+      <c r="E60">
+        <v>425.6</v>
+      </c>
+      <c r="F60">
+        <v>421.6</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B61">
+        <v>2579286</v>
+      </c>
+      <c r="C61">
+        <v>1216298</v>
+      </c>
+      <c r="E61">
+        <v>427</v>
+      </c>
+      <c r="F61">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B62">
+        <v>2579178</v>
+      </c>
+      <c r="C62">
+        <v>1216311</v>
+      </c>
+      <c r="E62">
+        <v>431</v>
+      </c>
+      <c r="F62">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B63">
+        <v>2578887</v>
+      </c>
+      <c r="C63">
+        <v>1216330</v>
+      </c>
+      <c r="E63">
+        <v>436</v>
+      </c>
+      <c r="F63">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B64">
+        <v>2578697</v>
+      </c>
+      <c r="C64">
+        <v>1216263</v>
+      </c>
+      <c r="E64">
+        <v>441</v>
+      </c>
+      <c r="F64">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B65">
+        <v>2578516</v>
+      </c>
+      <c r="C65">
+        <v>1216102</v>
+      </c>
+      <c r="E65">
+        <v>442</v>
+      </c>
+      <c r="F65">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B66">
+        <v>2578449</v>
+      </c>
+      <c r="C66">
+        <v>1216034</v>
+      </c>
+      <c r="E66">
+        <v>442.5</v>
+      </c>
+      <c r="F66">
+        <v>438.5</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B67">
+        <v>2578420</v>
+      </c>
+      <c r="C67">
+        <v>1216006</v>
+      </c>
+      <c r="E67">
+        <v>442.4</v>
+      </c>
+      <c r="F67">
+        <v>438.4</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B68">
+        <v>2578243</v>
+      </c>
+      <c r="C68">
+        <v>1215856</v>
+      </c>
+      <c r="E68">
+        <v>441.3</v>
+      </c>
+      <c r="F68">
+        <v>437.3</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B69">
+        <v>2578207</v>
+      </c>
+      <c r="C69">
+        <v>1215827</v>
+      </c>
+      <c r="E69">
+        <v>441</v>
+      </c>
+      <c r="F69">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B70">
+        <v>2578029</v>
+      </c>
+      <c r="C70">
+        <v>1215714</v>
+      </c>
+      <c r="E70">
+        <v>441.5</v>
+      </c>
+      <c r="F70">
+        <v>437.5</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B71">
+        <v>2577887</v>
+      </c>
+      <c r="C71">
+        <v>1215677</v>
+      </c>
+      <c r="E71">
+        <v>450.6</v>
+      </c>
+      <c r="F71">
+        <v>446.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update SS4 et SS2
Mise à jour des localisations SS2 et SS4. A ajouter dans le modèle hydraulique
</commit_message>
<xml_diff>
--- a/260508_Coord_nodes_SWMM.xlsx
+++ b/260508_Coord_nodes_SWMM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\ISSKA\Documents\GitHub\Twanntunnel_Hydraulic_SWMM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A585B224-074B-4281-A33D-F37B07E69FCB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A7DDACD-80A9-4666-920E-793FEE16A5EF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20385" windowHeight="11475" xr2:uid="{5560F17C-8740-4256-B354-A6A3ABF31B82}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="52">
   <si>
     <t>Holiloch_sonde</t>
   </si>
@@ -175,6 +175,12 @@
   </si>
   <si>
     <t>SonSto_SS4</t>
+  </si>
+  <si>
+    <t>SS2</t>
+  </si>
+  <si>
+    <t>SonSto_SS2</t>
   </si>
 </sst>
 </file>
@@ -529,7 +535,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{336D857F-22C8-4624-8585-90FCE8727574}">
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F73"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="43.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -789,10 +795,10 @@
         <v>27</v>
       </c>
       <c r="B19">
-        <v>2578252</v>
+        <v>2578260</v>
       </c>
       <c r="C19">
-        <v>1215886</v>
+        <v>1215897</v>
       </c>
       <c r="D19" t="s">
         <v>26</v>
@@ -1265,10 +1271,10 @@
         <v>49</v>
       </c>
       <c r="B53">
-        <v>2578254</v>
+        <v>2578262</v>
       </c>
       <c r="C53">
-        <v>1215885</v>
+        <v>1215896</v>
       </c>
       <c r="D53" t="s">
         <v>26</v>
@@ -1329,205 +1335,233 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="B60">
-        <v>2579848</v>
+        <v>2578291</v>
       </c>
       <c r="C60">
-        <v>1216615</v>
-      </c>
-      <c r="E60">
-        <v>425.6</v>
-      </c>
-      <c r="F60">
-        <v>421.6</v>
+        <v>1215937</v>
+      </c>
+      <c r="D60">
+        <v>446</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="B61">
-        <v>2579286</v>
+        <v>2578294</v>
       </c>
       <c r="C61">
-        <v>1216298</v>
-      </c>
-      <c r="E61">
-        <v>427</v>
-      </c>
-      <c r="F61">
-        <v>423</v>
+        <v>1215935</v>
+      </c>
+      <c r="D61">
+        <v>441.5</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B62">
-        <v>2579178</v>
+        <v>2579848</v>
       </c>
       <c r="C62">
-        <v>1216311</v>
+        <v>1216615</v>
       </c>
       <c r="E62">
-        <v>431</v>
+        <v>425.6</v>
       </c>
       <c r="F62">
-        <v>427</v>
+        <v>421.6</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B63">
-        <v>2578887</v>
+        <v>2579286</v>
       </c>
       <c r="C63">
-        <v>1216330</v>
+        <v>1216298</v>
       </c>
       <c r="E63">
-        <v>436</v>
+        <v>427</v>
       </c>
       <c r="F63">
-        <v>432</v>
+        <v>423</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B64">
-        <v>2578697</v>
+        <v>2579178</v>
       </c>
       <c r="C64">
-        <v>1216263</v>
+        <v>1216311</v>
       </c>
       <c r="E64">
-        <v>441</v>
+        <v>431</v>
       </c>
       <c r="F64">
-        <v>437</v>
+        <v>427</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B65">
-        <v>2578516</v>
+        <v>2578887</v>
       </c>
       <c r="C65">
-        <v>1216102</v>
+        <v>1216330</v>
       </c>
       <c r="E65">
-        <v>442</v>
+        <v>436</v>
       </c>
       <c r="F65">
-        <v>438</v>
+        <v>432</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B66">
-        <v>2578449</v>
+        <v>2578697</v>
       </c>
       <c r="C66">
-        <v>1216034</v>
+        <v>1216263</v>
       </c>
       <c r="E66">
-        <v>442.5</v>
+        <v>441</v>
       </c>
       <c r="F66">
-        <v>438.5</v>
+        <v>437</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B67">
-        <v>2578420</v>
+        <v>2578516</v>
       </c>
       <c r="C67">
-        <v>1216006</v>
+        <v>1216102</v>
       </c>
       <c r="E67">
-        <v>442.4</v>
+        <v>442</v>
       </c>
       <c r="F67">
-        <v>438.4</v>
+        <v>438</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B68">
-        <v>2578243</v>
+        <v>2578449</v>
       </c>
       <c r="C68">
-        <v>1215856</v>
+        <v>1216034</v>
       </c>
       <c r="E68">
-        <v>441.3</v>
+        <v>442.5</v>
       </c>
       <c r="F68">
-        <v>437.3</v>
+        <v>438.5</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B69">
-        <v>2578207</v>
+        <v>2578420</v>
       </c>
       <c r="C69">
-        <v>1215827</v>
+        <v>1216006</v>
       </c>
       <c r="E69">
-        <v>441</v>
+        <v>442.4</v>
       </c>
       <c r="F69">
-        <v>437</v>
+        <v>438.4</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B70">
-        <v>2578029</v>
+        <v>2578243</v>
       </c>
       <c r="C70">
-        <v>1215714</v>
+        <v>1215856</v>
       </c>
       <c r="E70">
-        <v>441.5</v>
+        <v>441.3</v>
       </c>
       <c r="F70">
-        <v>437.5</v>
+        <v>437.3</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B71">
+        <v>2578207</v>
+      </c>
+      <c r="C71">
+        <v>1215827</v>
+      </c>
+      <c r="E71">
+        <v>441</v>
+      </c>
+      <c r="F71">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B72">
+        <v>2578029</v>
+      </c>
+      <c r="C72">
+        <v>1215714</v>
+      </c>
+      <c r="E72">
+        <v>441.5</v>
+      </c>
+      <c r="F72">
+        <v>437.5</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B71">
+      <c r="B73">
         <v>2577887</v>
       </c>
-      <c r="C71">
+      <c r="C73">
         <v>1215677</v>
       </c>
-      <c r="E71">
+      <c r="E73">
         <v>450.6</v>
       </c>
-      <c r="F71">
+      <c r="F73">
         <v>446.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour coordonnées TWT
Les lignes en jaune sont les nodes qu'il faut considérer pour le TWT. Les longueur entre chaque node sont données sur la même ligne.
</commit_message>
<xml_diff>
--- a/260508_Coord_nodes_SWMM.xlsx
+++ b/260508_Coord_nodes_SWMM.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pierre-Yves\Documents\GitHub\Twanntunnel_Hydraulic_SWMM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\ISSKA\Documents\GitHub\Twanntunnel_Hydraulic_SWMM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C6DBF90-FCFA-4716-90CE-06B356E22E91}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC51DD34-F42A-4D81-A6F7-D7DDF8E0AB90}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20385" windowHeight="9060" xr2:uid="{5560F17C-8740-4256-B354-A6A3ABF31B82}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="57">
   <si>
     <t>Holiloch_sonde</t>
   </si>
@@ -114,9 +114,6 @@
     <t>SS1</t>
   </si>
   <si>
-    <t>TWT_Portail_Est</t>
-  </si>
-  <si>
     <t>Chaussée</t>
   </si>
   <si>
@@ -141,9 +138,6 @@
     <t>TWT_Branche_Est_Sonsto_60+540</t>
   </si>
   <si>
-    <t>TWT_Tschampet _60+650</t>
-  </si>
-  <si>
     <t>TWT_Fensterstollen_60+375</t>
   </si>
   <si>
@@ -184,6 +178,24 @@
   </si>
   <si>
     <t>Nouveaux nœuds</t>
+  </si>
+  <si>
+    <t>Longueur depuis portail Est:</t>
+  </si>
+  <si>
+    <t>TWT_PointHaut_60+650</t>
+  </si>
+  <si>
+    <t>TWT_Portail_Est_61+665</t>
+  </si>
+  <si>
+    <t>Longueur depuis  Point haut:</t>
+  </si>
+  <si>
+    <t>Longueur depuis  Fenster:</t>
+  </si>
+  <si>
+    <t>Longueur depuis  LiaisonLT</t>
   </si>
 </sst>
 </file>
@@ -199,12 +211,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -219,10 +237,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -538,7 +563,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{336D857F-22C8-4624-8585-90FCE8727574}">
-  <dimension ref="A1:I77"/>
+  <dimension ref="A1:J77"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="43.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -630,7 +655,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B7">
         <v>2578235</v>
@@ -658,7 +683,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B9">
         <v>2578239</v>
@@ -669,7 +694,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B10">
         <v>2578240</v>
@@ -1259,7 +1284,7 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B51">
         <v>2578260</v>
@@ -1273,7 +1298,7 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B52">
         <v>2578277</v>
@@ -1287,7 +1312,7 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B53">
         <v>2578262</v>
@@ -1301,7 +1326,7 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B54">
         <v>2578249</v>
@@ -1315,7 +1340,7 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
@@ -1365,10 +1390,10 @@
         <v>22</v>
       </c>
       <c r="E61" t="s">
+        <v>29</v>
+      </c>
+      <c r="F61" t="s">
         <v>30</v>
-      </c>
-      <c r="F61" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
@@ -1401,7 +1426,7 @@
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B64">
         <v>2578291</v>
@@ -1413,9 +1438,9 @@
         <v>446</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B65">
         <v>2578294</v>
@@ -1427,26 +1452,27 @@
         <v>441.5</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A66" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B66">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A66" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B66" s="3">
         <v>2579848</v>
       </c>
-      <c r="C66">
+      <c r="C66" s="3">
         <v>1216615</v>
       </c>
-      <c r="E66">
+      <c r="D66" s="3"/>
+      <c r="E66" s="3">
         <v>425.6</v>
       </c>
-      <c r="F66">
+      <c r="F66" s="3">
         <v>421.6</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B67">
         <v>2579286</v>
@@ -1461,9 +1487,9 @@
         <v>423</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B68">
         <v>2579178</v>
@@ -1478,9 +1504,9 @@
         <v>427</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B69">
         <v>2578887</v>
@@ -1495,9 +1521,9 @@
         <v>432</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B70">
         <v>2578697</v>
@@ -1512,9 +1538,9 @@
         <v>437</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B71">
         <v>2578516</v>
@@ -1529,26 +1555,33 @@
         <v>438</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A72" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B72">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A72" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B72" s="3">
         <v>2578449</v>
       </c>
-      <c r="C72">
+      <c r="C72" s="3">
         <v>1216034</v>
       </c>
-      <c r="E72">
+      <c r="D72" s="3"/>
+      <c r="E72" s="3">
         <v>442.5</v>
       </c>
-      <c r="F72">
+      <c r="F72" s="3">
         <v>438.5</v>
       </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I72" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J72">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B73">
         <v>2578420</v>
@@ -1563,26 +1596,33 @@
         <v>438.4</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A74" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B74">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A74" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B74" s="3">
         <v>2578243</v>
       </c>
-      <c r="C74">
+      <c r="C74" s="3">
         <v>1215856</v>
       </c>
-      <c r="E74">
+      <c r="D74" s="3"/>
+      <c r="E74" s="3">
         <v>441.3</v>
       </c>
-      <c r="F74">
+      <c r="F74" s="3">
         <v>437.3</v>
       </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="I74" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J74">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B75">
         <v>2578207</v>
@@ -1597,38 +1637,52 @@
         <v>437</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A76" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B76">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A76" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B76" s="3">
         <v>2578029</v>
       </c>
-      <c r="C76">
+      <c r="C76" s="3">
         <v>1215714</v>
       </c>
-      <c r="E76">
+      <c r="D76" s="3"/>
+      <c r="E76" s="3">
         <v>441.5</v>
       </c>
-      <c r="F76">
+      <c r="F76" s="3">
         <v>437.5</v>
       </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A77" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B77">
+      <c r="I76" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="J76">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A77" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B77" s="3">
         <v>2577887</v>
       </c>
-      <c r="C77">
+      <c r="C77" s="3">
         <v>1215677</v>
       </c>
-      <c r="E77">
+      <c r="D77" s="3"/>
+      <c r="E77" s="3">
         <v>450.6</v>
       </c>
-      <c r="F77">
+      <c r="F77" s="3">
         <v>446.5</v>
+      </c>
+      <c r="I77" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="J77">
+        <v>348</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Version 1 pour les simulations des phases
Il faudrait vérifier la cohérence des fichiers .inp et des deux fichiers excel avec les phases prévues. Ensuite on pourra lancer les simulations.
</commit_message>
<xml_diff>
--- a/260508_Coord_nodes_SWMM.xlsx
+++ b/260508_Coord_nodes_SWMM.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\ISSKA\Documents\GitHub\Twanntunnel_Hydraulic_SWMM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pierre-Yves\Documents\EPA SWMM Projects\Twann_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC51DD34-F42A-4D81-A6F7-D7DDF8E0AB90}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24A68AF4-79D5-4B41-8F2F-A96ED03FF144}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20385" windowHeight="9060" xr2:uid="{5560F17C-8740-4256-B354-A6A3ABF31B82}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20235" windowHeight="9060" xr2:uid="{5560F17C-8740-4256-B354-A6A3ABF31B82}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="63">
   <si>
     <t>Holiloch_sonde</t>
   </si>
@@ -196,6 +196,24 @@
   </si>
   <si>
     <t>Longueur depuis  LiaisonLT</t>
+  </si>
+  <si>
+    <t>Syst_Est_amont</t>
+  </si>
+  <si>
+    <t>Syst_Est_aval</t>
+  </si>
+  <si>
+    <t>Syst_Est_interm</t>
+  </si>
+  <si>
+    <t>TWT_Fensterstollen_aval_60+370</t>
+  </si>
+  <si>
+    <t>SonSto_F_sup</t>
+  </si>
+  <si>
+    <t>SonSto_porte</t>
   </si>
 </sst>
 </file>
@@ -237,7 +255,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -249,6 +267,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -563,7 +586,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{336D857F-22C8-4624-8585-90FCE8727574}">
-  <dimension ref="A1:J77"/>
+  <dimension ref="A1:J83"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="43.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -1014,7 +1037,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>4</v>
       </c>
@@ -1028,7 +1051,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>5</v>
       </c>
@@ -1042,7 +1065,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>6</v>
       </c>
@@ -1056,7 +1079,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>7</v>
       </c>
@@ -1070,7 +1093,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>6</v>
       </c>
@@ -1083,24 +1106,8 @@
       <c r="D37" t="s">
         <v>26</v>
       </c>
-      <c r="F37">
-        <f>B65-B64</f>
-        <v>3</v>
-      </c>
-      <c r="G37">
-        <f>C65-C64</f>
-        <v>-2</v>
-      </c>
-      <c r="H37">
-        <f>SQRT((F37*F37)+(G37*G37))</f>
-        <v>3.6055512754639891</v>
-      </c>
-      <c r="I37">
-        <f>SQRT((H37*H37)+(3.3*3.3))</f>
-        <v>4.8877397639399742</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>7</v>
       </c>
@@ -1114,7 +1121,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>8</v>
       </c>
@@ -1128,7 +1135,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>10</v>
       </c>
@@ -1142,7 +1149,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>8</v>
       </c>
@@ -1156,7 +1163,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>19</v>
       </c>
@@ -1170,7 +1177,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>9</v>
       </c>
@@ -1184,7 +1191,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>10</v>
       </c>
@@ -1198,7 +1205,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>20</v>
       </c>
@@ -1212,7 +1219,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>11</v>
       </c>
@@ -1226,7 +1233,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>12</v>
       </c>
@@ -1240,7 +1247,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>13</v>
       </c>
@@ -1254,7 +1261,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>14</v>
       </c>
@@ -1268,7 +1275,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>15</v>
       </c>
@@ -1282,7 +1289,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>41</v>
       </c>
@@ -1296,7 +1303,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>42</v>
       </c>
@@ -1310,7 +1317,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>47</v>
       </c>
@@ -1324,7 +1331,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>46</v>
       </c>
@@ -1334,16 +1341,13 @@
       <c r="C54">
         <v>1215879</v>
       </c>
-      <c r="D54" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>12</v>
       </c>
@@ -1357,7 +1361,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>14</v>
       </c>
@@ -1371,7 +1375,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <v>15</v>
       </c>
@@ -1385,307 +1389,421 @@
         <v>25</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A60" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B60">
+        <v>2578941.7599999998</v>
+      </c>
+      <c r="C60">
+        <v>1216615.48</v>
+      </c>
+      <c r="D60" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E61" t="s">
-        <v>29</v>
-      </c>
-      <c r="F61" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+        <v>59</v>
+      </c>
+      <c r="B61">
+        <v>2578918.5099999998</v>
+      </c>
+      <c r="C61">
+        <v>1216279.26</v>
+      </c>
+      <c r="D61" t="s">
+        <v>25</v>
+      </c>
+      <c r="F61" s="5">
+        <f>B61-B78</f>
+        <v>469.50999999977648</v>
+      </c>
+      <c r="G61" s="5">
+        <f>C61-C78</f>
+        <v>245.26000000000931</v>
+      </c>
+      <c r="H61">
+        <f>SQRT((F61*F61)+(G61*G61))</f>
+        <v>529.70945592824251</v>
+      </c>
+      <c r="I61">
+        <f>SQRT((H61*H61)+(3.3*3.3))</f>
+        <v>529.71973504844493</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B62">
-        <v>2578983</v>
-      </c>
-      <c r="C62">
-        <v>1216295</v>
-      </c>
-      <c r="D62">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A63" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B63">
-        <v>2578361</v>
-      </c>
-      <c r="C63">
-        <v>1215967</v>
-      </c>
-      <c r="D63">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A64" s="1" t="s">
-        <v>48</v>
+        <v>58</v>
+      </c>
+      <c r="B62" s="5">
+        <v>2578995.19</v>
+      </c>
+      <c r="C62" s="5">
+        <v>1216062.45</v>
+      </c>
+      <c r="D62" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A63" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B63" s="3">
+        <v>2578239</v>
+      </c>
+      <c r="C63" s="3">
+        <v>1215853</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E63" s="3">
+        <v>441</v>
+      </c>
+      <c r="F63" s="3">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A64" s="6" t="s">
+        <v>61</v>
       </c>
       <c r="B64">
-        <v>2578291</v>
+        <v>2578234</v>
       </c>
       <c r="C64">
-        <v>1215937</v>
-      </c>
-      <c r="D64">
-        <v>446</v>
-      </c>
+        <v>1215863</v>
+      </c>
+      <c r="D64" t="s">
+        <v>26</v>
+      </c>
+      <c r="E64" s="7"/>
+      <c r="F64" s="7"/>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A65" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B65">
-        <v>2578294</v>
-      </c>
-      <c r="C65">
-        <v>1215935</v>
-      </c>
-      <c r="D65">
-        <v>441.5</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A66" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B66" s="3">
-        <v>2579848</v>
-      </c>
-      <c r="C66" s="3">
-        <v>1216615</v>
-      </c>
-      <c r="D66" s="3"/>
-      <c r="E66" s="3">
-        <v>425.6</v>
-      </c>
-      <c r="F66" s="3">
-        <v>421.6</v>
-      </c>
+      <c r="A65" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B65" s="3">
+        <v>2578202</v>
+      </c>
+      <c r="C65" s="3">
+        <v>1215822</v>
+      </c>
+      <c r="D65" t="s">
+        <v>26</v>
+      </c>
+      <c r="E65" s="7"/>
+      <c r="F65" s="7"/>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B67">
-        <v>2579286</v>
-      </c>
-      <c r="C67">
-        <v>1216298</v>
-      </c>
-      <c r="E67">
-        <v>427</v>
-      </c>
-      <c r="F67">
-        <v>423</v>
+        <v>22</v>
+      </c>
+      <c r="E67" t="s">
+        <v>29</v>
+      </c>
+      <c r="F67" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="B68">
-        <v>2579178</v>
+        <v>2578983</v>
       </c>
       <c r="C68">
-        <v>1216311</v>
-      </c>
-      <c r="E68">
-        <v>431</v>
-      </c>
-      <c r="F68">
-        <v>427</v>
+        <v>1216295</v>
+      </c>
+      <c r="D68">
+        <v>436</v>
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B69">
-        <v>2578887</v>
+        <v>2578361</v>
       </c>
       <c r="C69">
-        <v>1216330</v>
-      </c>
-      <c r="E69">
-        <v>436</v>
-      </c>
-      <c r="F69">
-        <v>432</v>
+        <v>1215967</v>
+      </c>
+      <c r="D69">
+        <v>443</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="B70">
-        <v>2578697</v>
+        <v>2578291</v>
       </c>
       <c r="C70">
-        <v>1216263</v>
-      </c>
-      <c r="E70">
-        <v>441</v>
-      </c>
-      <c r="F70">
-        <v>437</v>
+        <v>1215937</v>
+      </c>
+      <c r="D70">
+        <v>446</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="B71">
-        <v>2578516</v>
+        <v>2578294</v>
       </c>
       <c r="C71">
-        <v>1216102</v>
-      </c>
-      <c r="E71">
-        <v>442</v>
-      </c>
-      <c r="F71">
-        <v>438</v>
+        <v>1215935</v>
+      </c>
+      <c r="D71">
+        <v>441.5</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B72" s="3">
-        <v>2578449</v>
+        <v>2579848</v>
       </c>
       <c r="C72" s="3">
-        <v>1216034</v>
+        <v>1216615</v>
       </c>
       <c r="D72" s="3"/>
       <c r="E72" s="3">
-        <v>442.5</v>
+        <v>425.6</v>
       </c>
       <c r="F72" s="3">
-        <v>438.5</v>
-      </c>
-      <c r="I72" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="J72">
-        <v>1015</v>
+        <v>421.6</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B73">
+        <v>2579286</v>
+      </c>
+      <c r="C73">
+        <v>1216298</v>
+      </c>
+      <c r="E73">
+        <v>427</v>
+      </c>
+      <c r="F73">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A74" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B74">
+        <v>2579178</v>
+      </c>
+      <c r="C74">
+        <v>1216311</v>
+      </c>
+      <c r="E74">
+        <v>431</v>
+      </c>
+      <c r="F74">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A75" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B75" s="3">
+        <v>2578887</v>
+      </c>
+      <c r="C75" s="3">
+        <v>1216330</v>
+      </c>
+      <c r="D75" s="3"/>
+      <c r="E75" s="3">
+        <v>436</v>
+      </c>
+      <c r="F75" s="3">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A76" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B76">
+        <v>2578697</v>
+      </c>
+      <c r="C76">
+        <v>1216263</v>
+      </c>
+      <c r="E76">
+        <v>441</v>
+      </c>
+      <c r="F76">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A77" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B77">
+        <v>2578516</v>
+      </c>
+      <c r="C77">
+        <v>1216102</v>
+      </c>
+      <c r="E77">
+        <v>442</v>
+      </c>
+      <c r="F77">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A78" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B78" s="3">
+        <v>2578449</v>
+      </c>
+      <c r="C78" s="3">
+        <v>1216034</v>
+      </c>
+      <c r="D78" s="3"/>
+      <c r="E78" s="3">
+        <v>442.5</v>
+      </c>
+      <c r="F78" s="3">
+        <v>438.5</v>
+      </c>
+      <c r="I78" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="J78">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A79" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B73">
+      <c r="B79" s="3">
         <v>2578420</v>
       </c>
-      <c r="C73">
+      <c r="C79" s="3">
         <v>1216006</v>
       </c>
-      <c r="E73">
+      <c r="D79" s="3"/>
+      <c r="E79" s="3">
         <v>442.4</v>
       </c>
-      <c r="F73">
+      <c r="F79" s="3">
         <v>438.4</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A74" s="2" t="s">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A80" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B74" s="3">
+      <c r="B80" s="3">
         <v>2578243</v>
       </c>
-      <c r="C74" s="3">
+      <c r="C80" s="3">
         <v>1215856</v>
       </c>
-      <c r="D74" s="3"/>
-      <c r="E74" s="3">
+      <c r="D80" s="3"/>
+      <c r="E80" s="3">
         <v>441.3</v>
       </c>
-      <c r="F74" s="3">
+      <c r="F80" s="3">
         <v>437.3</v>
       </c>
-      <c r="I74" s="4" t="s">
+      <c r="I80" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="J74">
+      <c r="J80">
         <v>275</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A75" s="1" t="s">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A81" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B75">
+      <c r="B81" s="3">
         <v>2578207</v>
       </c>
-      <c r="C75">
+      <c r="C81" s="3">
         <v>1215827</v>
       </c>
-      <c r="E75">
+      <c r="D81" s="3"/>
+      <c r="E81" s="3">
         <v>441</v>
       </c>
-      <c r="F75">
+      <c r="F81" s="3">
         <v>437</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A76" s="2" t="s">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A82" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B76" s="3">
+      <c r="B82" s="3">
         <v>2578029</v>
       </c>
-      <c r="C76" s="3">
+      <c r="C82" s="3">
         <v>1215714</v>
       </c>
-      <c r="D76" s="3"/>
-      <c r="E76" s="3">
+      <c r="D82" s="3"/>
+      <c r="E82" s="3">
         <v>441.5</v>
       </c>
-      <c r="F76" s="3">
+      <c r="F82" s="3">
         <v>437.5</v>
       </c>
-      <c r="I76" s="4" t="s">
+      <c r="I82" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="J76">
+      <c r="J82">
         <v>265</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A77" s="2" t="s">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A83" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B77" s="3">
+      <c r="B83" s="3">
         <v>2577887</v>
       </c>
-      <c r="C77" s="3">
+      <c r="C83" s="3">
         <v>1215677</v>
       </c>
-      <c r="D77" s="3"/>
-      <c r="E77" s="3">
+      <c r="D83" s="3"/>
+      <c r="E83" s="3">
         <v>450.6</v>
       </c>
-      <c r="F77" s="3">
+      <c r="F83" s="3">
         <v>446.5</v>
       </c>
-      <c r="I77" s="4" t="s">
+      <c r="I83" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="J77">
+      <c r="J83">
         <v>348</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>